<commit_message>
Save all new file changes and updates
</commit_message>
<xml_diff>
--- a/sample_data/Medication Error3.xlsx
+++ b/sample_data/Medication Error3.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="V:\Tobesaved\indicators\المؤشرات في مجلس الادارة\تحليل المؤشرات\d hazimeh\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\healthcare_motality_system\sample_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -5015,9 +5015,7 @@
               </c:spPr>
             </c:leaderLines>
             <c:extLst>
-              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
-                <c15:layout/>
-              </c:ext>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
           </c:dLbls>
           <c:cat>
@@ -5083,7 +5081,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -10123,21 +10120,21 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:R39"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="16.140625" style="58" customWidth="1"/>
-    <col min="2" max="2" width="8.5703125" style="86" customWidth="1"/>
-    <col min="3" max="4" width="4.42578125" style="59" customWidth="1"/>
+    <col min="1" max="1" width="16.109375" style="58" customWidth="1"/>
+    <col min="2" max="2" width="8.5546875" style="86" customWidth="1"/>
+    <col min="3" max="4" width="4.44140625" style="59" customWidth="1"/>
     <col min="5" max="5" width="12" style="58" customWidth="1"/>
-    <col min="6" max="6" width="4.42578125" style="60" customWidth="1"/>
-    <col min="7" max="9" width="14.85546875" style="58" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" style="87" customWidth="1"/>
-    <col min="11" max="11" width="13.85546875" style="58" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" style="58" customWidth="1"/>
-    <col min="13" max="14" width="3.85546875" style="58" customWidth="1"/>
+    <col min="6" max="6" width="4.44140625" style="60" customWidth="1"/>
+    <col min="7" max="9" width="14.88671875" style="58" customWidth="1"/>
+    <col min="10" max="10" width="14.88671875" style="87" customWidth="1"/>
+    <col min="11" max="11" width="13.88671875" style="58" customWidth="1"/>
+    <col min="12" max="12" width="15.6640625" style="58" customWidth="1"/>
+    <col min="13" max="14" width="3.88671875" style="58" customWidth="1"/>
     <col min="15" max="15" width="13" style="58" customWidth="1"/>
     <col min="16" max="16" width="30" style="61" customWidth="1"/>
-    <col min="17" max="17" width="44.42578125" style="58" customWidth="1"/>
+    <col min="17" max="17" width="44.44140625" style="58" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="84" customHeight="1">
@@ -10196,7 +10193,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="72">
+    <row r="2" spans="1:18" ht="52.8">
       <c r="A2" s="88" t="s">
         <v>349</v>
       </c>
@@ -10244,7 +10241,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" ht="90">
+    <row r="3" spans="1:18" ht="66">
       <c r="A3" s="88" t="s">
         <v>349</v>
       </c>
@@ -10292,7 +10289,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:18" ht="45">
+    <row r="4" spans="1:18" ht="46.8">
       <c r="A4" s="88" t="s">
         <v>349</v>
       </c>
@@ -10340,7 +10337,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:18" ht="90">
+    <row r="5" spans="1:18" ht="66">
       <c r="A5" s="88" t="s">
         <v>349</v>
       </c>
@@ -10388,7 +10385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="72">
+    <row r="6" spans="1:18" ht="46.8">
       <c r="A6" s="88" t="s">
         <v>349</v>
       </c>
@@ -10436,7 +10433,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="108">
+    <row r="7" spans="1:18" ht="79.2">
       <c r="A7" s="88" t="s">
         <v>349</v>
       </c>
@@ -10484,7 +10481,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:18" ht="72">
+    <row r="8" spans="1:18" ht="52.8">
       <c r="A8" s="88" t="s">
         <v>349</v>
       </c>
@@ -10532,7 +10529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="54">
+    <row r="9" spans="1:18" ht="51">
       <c r="A9" s="88" t="s">
         <v>349</v>
       </c>
@@ -10580,7 +10577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:18" ht="90">
+    <row r="10" spans="1:18" ht="66">
       <c r="A10" s="88" t="s">
         <v>349</v>
       </c>
@@ -10628,7 +10625,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:18" ht="54">
+    <row r="11" spans="1:18" ht="51">
       <c r="A11" s="88" t="s">
         <v>349</v>
       </c>
@@ -10676,7 +10673,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:18" ht="126">
+    <row r="12" spans="1:18" ht="92.4">
       <c r="A12" s="88" t="s">
         <v>349</v>
       </c>
@@ -10724,7 +10721,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:18" ht="72">
+    <row r="13" spans="1:18" ht="52.8">
       <c r="A13" s="88" t="s">
         <v>349</v>
       </c>
@@ -10772,7 +10769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:18" ht="90">
+    <row r="14" spans="1:18" ht="66">
       <c r="A14" s="88" t="s">
         <v>349</v>
       </c>
@@ -10820,7 +10817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="54">
+    <row r="15" spans="1:18" ht="46.8">
       <c r="A15" s="88" t="s">
         <v>349</v>
       </c>
@@ -10866,7 +10863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:18" ht="90">
+    <row r="16" spans="1:18" ht="66">
       <c r="A16" s="88" t="s">
         <v>349</v>
       </c>
@@ -10914,7 +10911,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:18" ht="54">
+    <row r="17" spans="1:18" ht="51">
       <c r="A17" s="88" t="s">
         <v>349</v>
       </c>
@@ -10962,7 +10959,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:18" ht="54">
+    <row r="18" spans="1:18" ht="46.8">
       <c r="A18" s="88" t="s">
         <v>349</v>
       </c>
@@ -11010,7 +11007,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="90">
+    <row r="19" spans="1:18" ht="66">
       <c r="A19" s="88" t="s">
         <v>349</v>
       </c>
@@ -11058,7 +11055,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:18" ht="56.25">
+    <row r="20" spans="1:18" ht="52.2">
       <c r="A20" s="89" t="s">
         <v>236</v>
       </c>
@@ -11106,7 +11103,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:18" ht="56.25">
+    <row r="21" spans="1:18" ht="52.2">
       <c r="A21" s="89" t="s">
         <v>236</v>
       </c>
@@ -11154,7 +11151,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:18" ht="55.5">
+    <row r="22" spans="1:18" ht="43.2">
       <c r="A22" s="68" t="s">
         <v>235</v>
       </c>
@@ -11204,7 +11201,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:18" ht="55.5">
+    <row r="23" spans="1:18" ht="46.8">
       <c r="A23" s="68" t="s">
         <v>235</v>
       </c>
@@ -11252,7 +11249,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="55.5">
+    <row r="24" spans="1:18" ht="43.2">
       <c r="A24" s="68" t="s">
         <v>235</v>
       </c>
@@ -11302,7 +11299,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:18" ht="54.75">
+    <row r="25" spans="1:18" ht="48.6">
       <c r="A25" s="68" t="s">
         <v>235</v>
       </c>
@@ -11350,7 +11347,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="54">
+    <row r="26" spans="1:18" ht="48.6">
       <c r="A26" s="68" t="s">
         <v>235</v>
       </c>
@@ -11400,7 +11397,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="54">
+    <row r="27" spans="1:18" ht="48.6">
       <c r="A27" s="68" t="s">
         <v>235</v>
       </c>
@@ -11448,7 +11445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="54">
+    <row r="28" spans="1:18" ht="48.6">
       <c r="A28" s="68" t="s">
         <v>235</v>
       </c>
@@ -11496,7 +11493,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:18" ht="54.75">
+    <row r="29" spans="1:18" ht="43.2">
       <c r="A29" s="68" t="s">
         <v>235</v>
       </c>
@@ -11546,7 +11543,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="54.75">
+    <row r="30" spans="1:18" ht="43.2">
       <c r="A30" s="68" t="s">
         <v>235</v>
       </c>
@@ -11596,7 +11593,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="55.5">
+    <row r="31" spans="1:18" ht="43.2">
       <c r="A31" s="68" t="s">
         <v>235</v>
       </c>
@@ -11644,7 +11641,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:18" ht="54">
+    <row r="32" spans="1:18" ht="48.6">
       <c r="A32" s="68" t="s">
         <v>235</v>
       </c>
@@ -11694,7 +11691,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:18" ht="36">
+    <row r="33" spans="1:18" ht="26.4">
       <c r="A33" s="68" t="s">
         <v>413</v>
       </c>
@@ -11742,7 +11739,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:18" ht="54.75">
+    <row r="34" spans="1:18" ht="48.6">
       <c r="A34" s="68" t="s">
         <v>235</v>
       </c>
@@ -11790,7 +11787,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="54">
+    <row r="35" spans="1:18" ht="48.6">
       <c r="A35" s="96" t="s">
         <v>235</v>
       </c>
@@ -11840,7 +11837,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:18" ht="72">
+    <row r="36" spans="1:18" ht="52.8">
       <c r="A36" s="96" t="s">
         <v>235</v>
       </c>
@@ -11890,7 +11887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:18" ht="54">
+    <row r="37" spans="1:18" ht="48.6">
       <c r="A37" s="68" t="s">
         <v>235</v>
       </c>
@@ -11938,7 +11935,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:18" ht="54.75">
+    <row r="38" spans="1:18" ht="48.6">
       <c r="A38" s="68" t="s">
         <v>235</v>
       </c>
@@ -12003,10 +12000,10 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A2:B34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="83.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="83.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:2">
@@ -12194,12 +12191,12 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A42"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="107.42578125" customWidth="1"/>
-    <col min="2" max="2" width="36.85546875" customWidth="1"/>
-    <col min="3" max="3" width="37.7109375" customWidth="1"/>
-    <col min="4" max="4" width="35.42578125" customWidth="1"/>
+    <col min="1" max="1" width="107.44140625" customWidth="1"/>
+    <col min="2" max="2" width="36.88671875" customWidth="1"/>
+    <col min="3" max="3" width="37.6640625" customWidth="1"/>
+    <col min="4" max="4" width="35.44140625" customWidth="1"/>
     <col min="8" max="8" width="27" customWidth="1"/>
   </cols>
   <sheetData>
@@ -12313,47 +12310,47 @@
         <v>9</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="15.75">
+    <row r="23" spans="1:1" ht="15.6">
       <c r="A23" s="26" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="15.75">
+    <row r="24" spans="1:1" ht="15.6">
       <c r="A24" s="26" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="15.75">
+    <row r="25" spans="1:1" ht="15.6">
       <c r="A25" s="26" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="15.75">
+    <row r="26" spans="1:1" ht="15.6">
       <c r="A26" s="26" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="15.75">
+    <row r="27" spans="1:1" ht="15.6">
       <c r="A27" s="26" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="15.75">
+    <row r="28" spans="1:1" ht="15.6">
       <c r="A28" s="26" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="15.75">
+    <row r="29" spans="1:1" ht="15.6">
       <c r="A29" s="26" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="15.75">
+    <row r="30" spans="1:1" ht="15.6">
       <c r="A30" s="26" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="15.75">
+    <row r="31" spans="1:1" ht="15.6">
       <c r="A31" s="26" t="s">
         <v>141</v>
       </c>
@@ -12403,10 +12400,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="19.5">
+    <row r="41" spans="1:1">
       <c r="A41" s="28"/>
     </row>
-    <row r="42" spans="1:1" ht="19.5">
+    <row r="42" spans="1:1">
       <c r="A42" s="7"/>
     </row>
   </sheetData>
@@ -12417,66 +12414,66 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="82.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="66.28515625" customWidth="1"/>
+    <col min="1" max="1" width="82.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="66.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="21.75">
+    <row r="1" spans="1:4">
       <c r="A1" s="18" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="21.75">
+    <row r="2" spans="1:4">
       <c r="A2" s="17" t="s">
         <v>152</v>
       </c>
       <c r="D2" s="13"/>
     </row>
-    <row r="3" spans="1:4" ht="21.75">
+    <row r="3" spans="1:4">
       <c r="A3" s="17" t="s">
         <v>145</v>
       </c>
       <c r="D3" s="13"/>
     </row>
-    <row r="4" spans="1:4" ht="21.75">
+    <row r="4" spans="1:4">
       <c r="A4" s="17" t="s">
         <v>146</v>
       </c>
       <c r="D4" s="13"/>
     </row>
-    <row r="5" spans="1:4" ht="21.75">
+    <row r="5" spans="1:4">
       <c r="A5" s="17" t="s">
         <v>147</v>
       </c>
       <c r="D5" s="13"/>
     </row>
-    <row r="6" spans="1:4" ht="21.75">
+    <row r="6" spans="1:4">
       <c r="A6" s="17" t="s">
         <v>148</v>
       </c>
       <c r="D6" s="13"/>
     </row>
-    <row r="7" spans="1:4" ht="21.75">
+    <row r="7" spans="1:4">
       <c r="A7" s="17" t="s">
         <v>67</v>
       </c>
       <c r="D7" s="13"/>
     </row>
-    <row r="8" spans="1:4" ht="21.75">
+    <row r="8" spans="1:4">
       <c r="A8" s="17" t="s">
         <v>149</v>
       </c>
       <c r="D8" s="13"/>
     </row>
-    <row r="9" spans="1:4" ht="21.75">
+    <row r="9" spans="1:4">
       <c r="A9" s="17" t="s">
         <v>150</v>
       </c>
       <c r="D9" s="13"/>
     </row>
-    <row r="10" spans="1:4" ht="21.75">
+    <row r="10" spans="1:4">
       <c r="A10" s="5" t="s">
         <v>151</v>
       </c>
@@ -12489,54 +12486,54 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="76.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="76.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30">
+    <row r="1" spans="1:4" ht="21">
       <c r="A1" s="32" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="30">
+    <row r="2" spans="1:4" ht="21">
       <c r="A2" s="33" t="s">
         <v>155</v>
       </c>
       <c r="D2" s="19"/>
     </row>
-    <row r="3" spans="1:4" ht="27.75">
+    <row r="3" spans="1:4" ht="20.399999999999999">
       <c r="A3" s="34" t="s">
         <v>153</v>
       </c>
       <c r="D3" s="19"/>
     </row>
-    <row r="4" spans="1:4" ht="27.75">
+    <row r="4" spans="1:4" ht="20.399999999999999">
       <c r="A4" s="34" t="s">
         <v>154</v>
       </c>
       <c r="D4" s="19"/>
     </row>
-    <row r="5" spans="1:4" ht="27.75">
+    <row r="5" spans="1:4" ht="20.399999999999999">
       <c r="A5" s="34" t="s">
         <v>42</v>
       </c>
       <c r="D5" s="19"/>
     </row>
-    <row r="6" spans="1:4" ht="27.75">
+    <row r="6" spans="1:4" ht="20.399999999999999">
       <c r="A6" s="35" t="s">
         <v>43</v>
       </c>
       <c r="D6" s="19"/>
     </row>
-    <row r="7" spans="1:4" ht="27.75">
+    <row r="7" spans="1:4" ht="20.399999999999999">
       <c r="A7" s="35" t="s">
         <v>44</v>
       </c>
       <c r="D7" s="19"/>
     </row>
-    <row r="8" spans="1:4" ht="27.75">
+    <row r="8" spans="1:4" ht="20.399999999999999">
       <c r="A8" s="36" t="s">
         <v>156</v>
       </c>
@@ -12554,7 +12551,7 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="55" customWidth="1"/>
   </cols>
@@ -12687,9 +12684,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="27.5703125" customWidth="1"/>
+    <col min="1" max="1" width="27.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -12730,7 +12727,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
   </cols>
@@ -12819,9 +12816,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="25.42578125" customWidth="1"/>
+    <col min="1" max="1" width="25.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -12834,27 +12831,27 @@
         <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="18">
+    <row r="3" spans="1:1">
       <c r="A3" s="1" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="18">
+    <row r="4" spans="1:1">
       <c r="A4" s="1" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="18">
+    <row r="5" spans="1:1">
       <c r="A5" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="18">
+    <row r="6" spans="1:1">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="18">
+    <row r="7" spans="1:1">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
@@ -12867,10 +12864,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="21.28515625" customWidth="1"/>
-    <col min="2" max="2" width="21.140625" customWidth="1"/>
+    <col min="1" max="1" width="21.33203125" customWidth="1"/>
+    <col min="2" max="2" width="21.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -12881,7 +12878,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="21.75">
+    <row r="2" spans="1:2">
       <c r="A2" s="14" t="s">
         <v>64</v>
       </c>
@@ -12889,7 +12886,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="21.75">
+    <row r="3" spans="1:2">
       <c r="A3" s="14" t="s">
         <v>65</v>
       </c>
@@ -12897,7 +12894,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="21.75">
+    <row r="4" spans="1:2">
       <c r="A4" s="14" t="s">
         <v>66</v>
       </c>
@@ -12913,176 +12910,176 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:A34"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="28.7109375" customWidth="1"/>
-    <col min="3" max="3" width="7.5703125" customWidth="1"/>
-    <col min="6" max="6" width="23.28515625" customWidth="1"/>
-    <col min="7" max="7" width="37.28515625" customWidth="1"/>
+    <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.6640625" customWidth="1"/>
+    <col min="3" max="3" width="7.5546875" customWidth="1"/>
+    <col min="6" max="6" width="23.33203125" customWidth="1"/>
+    <col min="7" max="7" width="37.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="21.75">
+    <row r="1" spans="1:1">
       <c r="A1" s="47" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="19.5">
+    <row r="2" spans="1:1">
       <c r="A2" s="48" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="19.5">
+    <row r="3" spans="1:1">
       <c r="A3" s="48" t="s">
         <v>212</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="19.5">
+    <row r="4" spans="1:1">
       <c r="A4" s="48" t="s">
         <v>213</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="19.5">
+    <row r="5" spans="1:1">
       <c r="A5" s="48" t="s">
         <v>217</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="19.5">
+    <row r="6" spans="1:1">
       <c r="A6" s="48" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="19.5">
+    <row r="7" spans="1:1">
       <c r="A7" s="48" t="s">
         <v>215</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="19.5">
+    <row r="8" spans="1:1">
       <c r="A8" s="48" t="s">
         <v>216</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="19.5">
+    <row r="9" spans="1:1">
       <c r="A9" s="48" t="s">
         <v>218</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="19.5">
+    <row r="10" spans="1:1">
       <c r="A10" s="48" t="s">
         <v>219</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="19.5">
+    <row r="11" spans="1:1">
       <c r="A11" s="48" t="s">
         <v>208</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="19.5">
+    <row r="12" spans="1:1">
       <c r="A12" s="48" t="s">
         <v>220</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="19.5">
+    <row r="13" spans="1:1">
       <c r="A13" s="48" t="s">
         <v>209</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="19.5">
+    <row r="14" spans="1:1">
       <c r="A14" s="48" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="19.5">
+    <row r="15" spans="1:1">
       <c r="A15" s="48" t="s">
         <v>221</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="19.5">
+    <row r="16" spans="1:1">
       <c r="A16" s="48" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="19.5">
+    <row r="17" spans="1:1">
       <c r="A17" s="48" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="19.5">
+    <row r="18" spans="1:1">
       <c r="A18" s="48" t="s">
         <v>210</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="19.5">
+    <row r="19" spans="1:1">
       <c r="A19" s="48" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="19.5">
+    <row r="20" spans="1:1">
       <c r="A20" s="48" t="s">
         <v>223</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="19.5">
+    <row r="21" spans="1:1">
       <c r="A21" s="48" t="s">
         <v>224</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="19.5">
+    <row r="22" spans="1:1">
       <c r="A22" s="48" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="19.5">
+    <row r="23" spans="1:1">
       <c r="A23" s="48" t="s">
         <v>226</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="19.5">
+    <row r="24" spans="1:1">
       <c r="A24" s="48" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="19.5">
+    <row r="25" spans="1:1">
       <c r="A25" s="46" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="19.5">
+    <row r="26" spans="1:1">
       <c r="A26" s="46" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="19.5">
+    <row r="27" spans="1:1">
       <c r="A27" s="46" t="s">
         <v>227</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="19.5">
+    <row r="28" spans="1:1" ht="20.399999999999999">
       <c r="A28" s="46" t="s">
         <v>205</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="19.5">
+    <row r="29" spans="1:1">
       <c r="A29" s="46" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="19.5">
+    <row r="30" spans="1:1" ht="20.399999999999999">
       <c r="A30" s="46" t="s">
         <v>206</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="19.5">
+    <row r="31" spans="1:1" ht="20.399999999999999">
       <c r="A31" s="46" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="19.5">
+    <row r="32" spans="1:1">
       <c r="A32" s="46" t="s">
         <v>228</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="19.5">
+    <row r="33" spans="1:1">
       <c r="A33" s="46" t="s">
         <v>30</v>
       </c>
@@ -13099,9 +13096,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="32.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="32.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26" customWidth="1"/>
   </cols>
   <sheetData>
@@ -13113,52 +13110,52 @@
         <v>182</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="19.5">
+    <row r="2" spans="1:2">
       <c r="A2" s="4" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="19.5">
+    <row r="3" spans="1:2">
       <c r="A3" s="4" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="19.5">
+    <row r="4" spans="1:2">
       <c r="A4" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="19.5">
+    <row r="5" spans="1:2">
       <c r="A5" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="19.5">
+    <row r="6" spans="1:2">
       <c r="A6" s="4" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="19.5">
+    <row r="7" spans="1:2">
       <c r="A7" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="19.5">
+    <row r="8" spans="1:2">
       <c r="A8" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="19.5">
+    <row r="9" spans="1:2">
       <c r="A9" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:2" ht="19.5">
+    <row r="10" spans="1:2">
       <c r="A10" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="19.5">
+    <row r="11" spans="1:2">
       <c r="A11" s="5" t="s">
         <v>33</v>
       </c>
@@ -13171,11 +13168,11 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="29" customWidth="1"/>
-    <col min="2" max="2" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="22.42578125" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="27" customHeight="1">
@@ -13191,7 +13188,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="20.25">
+    <row r="4" spans="1:3" ht="15">
       <c r="A4" s="8" t="s">
         <v>45</v>
       </c>
@@ -13200,7 +13197,7 @@
       </c>
       <c r="C4" s="19"/>
     </row>
-    <row r="5" spans="1:3" ht="20.25">
+    <row r="5" spans="1:3" ht="15">
       <c r="A5" s="8" t="s">
         <v>46</v>
       </c>
@@ -13209,7 +13206,7 @@
       </c>
       <c r="C5" s="19"/>
     </row>
-    <row r="6" spans="1:3" ht="20.25">
+    <row r="6" spans="1:3" ht="15">
       <c r="A6" s="8" t="s">
         <v>47</v>
       </c>
@@ -13218,7 +13215,7 @@
       </c>
       <c r="C6" s="19"/>
     </row>
-    <row r="7" spans="1:3" ht="20.25">
+    <row r="7" spans="1:3" ht="15">
       <c r="A7" s="8" t="s">
         <v>48</v>
       </c>
@@ -13227,7 +13224,7 @@
       </c>
       <c r="C7" s="19"/>
     </row>
-    <row r="8" spans="1:3" ht="20.25">
+    <row r="8" spans="1:3" ht="15">
       <c r="A8" s="9" t="s">
         <v>49</v>
       </c>
@@ -13236,7 +13233,7 @@
       </c>
       <c r="C8" s="19"/>
     </row>
-    <row r="9" spans="1:3" ht="20.25">
+    <row r="9" spans="1:3" ht="15">
       <c r="A9" s="9" t="s">
         <v>50</v>
       </c>
@@ -13244,7 +13241,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="20.25">
+    <row r="10" spans="1:3" ht="15">
       <c r="A10" s="10" t="s">
         <v>51</v>
       </c>
@@ -13253,7 +13250,7 @@
       </c>
       <c r="C10" s="19"/>
     </row>
-    <row r="11" spans="1:3" ht="20.25">
+    <row r="11" spans="1:3" ht="15">
       <c r="A11" s="10" t="s">
         <v>52</v>
       </c>
@@ -13262,7 +13259,7 @@
       </c>
       <c r="C11" s="19"/>
     </row>
-    <row r="12" spans="1:3" ht="20.25">
+    <row r="12" spans="1:3" ht="15">
       <c r="A12" s="10" t="s">
         <v>53</v>
       </c>
@@ -13271,7 +13268,7 @@
       </c>
       <c r="C12" s="19"/>
     </row>
-    <row r="13" spans="1:3" ht="20.25">
+    <row r="13" spans="1:3" ht="15">
       <c r="A13" s="10" t="s">
         <v>54</v>
       </c>
@@ -13280,17 +13277,17 @@
       </c>
       <c r="C13" s="19"/>
     </row>
-    <row r="14" spans="1:3" ht="20.25">
+    <row r="14" spans="1:3" ht="15">
       <c r="A14" s="10" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="20.25">
+    <row r="15" spans="1:3" ht="15.6">
       <c r="A15" s="11" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="20.25">
+    <row r="16" spans="1:3" ht="15.6">
       <c r="A16" s="11" t="s">
         <v>57</v>
       </c>
@@ -13304,13 +13301,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:F97"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33.85546875" customWidth="1"/>
-    <col min="2" max="2" width="14.5703125" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="13.5703125" customWidth="1"/>
-    <col min="6" max="6" width="12.140625" customWidth="1"/>
+    <col min="1" max="1" width="33.88671875" customWidth="1"/>
+    <col min="2" max="2" width="14.5546875" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="13.5546875" customWidth="1"/>
+    <col min="6" max="6" width="12.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -13773,7 +13770,7 @@
         <v>0.28888888888888886</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="30">
+    <row r="58" spans="1:5" ht="28.8">
       <c r="A58" s="115" t="s">
         <v>324</v>
       </c>
@@ -14082,7 +14079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="30">
+    <row r="85" spans="1:6" ht="28.8">
       <c r="A85" s="116" t="s">
         <v>410</v>
       </c>

</xml_diff>